<commit_message>
Corrige RO65 para R$60 (info do Jonathan, não R$250)
O custo do kit RO65 unitário é R$60 — a planilha estava certa, eu havia
guardado R$250 por engano. Atualizado em materiais.json, no app
(validacao-orcamento.html), nas notas e no orçamento da Camila (material
cai p/ R$12.858, investimento sugerido MC38% ~R$47.455).

https://claude.ai/code/session_01KBgdwSXG3nucLVLi4YZwtE
</commit_message>
<xml_diff>
--- a/.claude/skills/orcamentista-marcenaria/projetos/orcamento-camila-lavinia.xlsx
+++ b/.claude/skills/orcamentista-marcenaria/projetos/orcamento-camila-lavinia.xlsx
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="B9" s="19" t="n">
-        <v>49270</v>
+        <v>47460</v>
       </c>
       <c r="D9" s="102" t="n"/>
       <c r="F9" s="21" t="n"/>
@@ -2578,7 +2578,7 @@
         <v>3</v>
       </c>
       <c r="C100" s="97" t="n">
-        <v>250</v>
+        <v>60</v>
       </c>
       <c r="D100" s="91">
         <f>SUM(B100*C100)</f>

</xml_diff>